<commit_message>
Test plan: paired-test rule, judge-first gate, fallback branch
</commit_message>
<xml_diff>
--- a/Test_Plani.xlsx
+++ b/Test_Plani.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Özet" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Planı'!$A$4:$I$46</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Planı'!$A$4:$I$47</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="174">
   <si>
     <t xml:space="preserve">Collections Builder — Test Planı ve Karar Kuralları</t>
   </si>
   <si>
-    <t xml:space="preserve">Gürültü = baseline 3 kez koşturulunca ölçülen 2×SD. Sarı sütunlar ekip tarafından doldurulur (Durum açılır listeden).</t>
+    <t xml:space="preserve">Kazanç = eşleştirilmiş case bazında testte p&lt;0.1 ve kritik case tiplerinde düşüş yok (aggregate 2×SD kullanılmaz). Sarı sütunlar ekip tarafından doldurulur (Durum açılır listeden).</t>
   </si>
   <si>
     <t xml:space="preserve">Bölüm</t>
@@ -60,54 +60,81 @@
     <t xml:space="preserve">Not</t>
   </si>
   <si>
+    <t xml:space="preserve">0. Ön koşul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collections domain klasörü</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kickoff'tan önce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2–3 sahte brief, 7 tool + mock veri, 16 case tipi persona kütüphanesi, 4 kritik an unit testi hazır</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hazır değilse hiçbir test koşamaz; önce bu tamamlanır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bekliyor</t>
+  </si>
+  <si>
     <t xml:space="preserve">0. Önce ölçülecekler</t>
   </si>
   <si>
     <t xml:space="preserve">T0.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Baseline × 3</t>
+    <t xml:space="preserve">Practice baseline × 3</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
   </si>
   <si>
-    <t xml:space="preserve">2×SD = gürültü eşiği</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bu eşiğin altındaki hiçbir farka “kazanç” denmez.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bekliyor</t>
+    <t xml:space="preserve">Case başına run-to-run varyansı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayrıştıran case seti ve eşleştirilmiş test için temel. Cache'lenir.</t>
   </si>
   <si>
     <t xml:space="preserve">T0.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Lokal yargıç ile Freya verdict uyumu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥ %85</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lokal simülatör iç döngü olur, Freya yalnızca onaylar. GEPA açılır.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">%70–85</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lokal yalnızca bariz kötüleri eler; sıralama Freya'da yapılır.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt; %70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lokal yargıç bırakılır, yalnızca Freya verdict'i kullanılır. GEPA iptal.</t>
+    <t xml:space="preserve">Yargıç düzeltmesi (uyumdan önce)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool-call log verilir; eylemler sözlerden ayrı, evet/hayır sorular, sıcaklık 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uyum bu düzeltmeden sonra ölçülür.</t>
   </si>
   <si>
     <t xml:space="preserve">T0.3</t>
   </si>
   <si>
+    <t xml:space="preserve">Lokal yargıç ile Freya verdict uyumu (case tipi bazında)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">İlk practice verdict'leri dönünce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ %85 genelde VE üçüncü şahıs / doğrulama / söz verme case'lerinde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lokal simülatör iç döngü olur, Freya yalnızca onaylar. Bölüm 3–4 açılır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bunun altında</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALLBACK: Bölüm 3'ün simülasyonlu kısımları ve bölüm 4 düşer. Sadece Freya: builder-prompt düzeltmeleri + dersler kütüphanesi + eşleştirilmiş test. Lokal yargıç dev triage için kalır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T0.4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unit test skoru ile Freya skoru sıralaması (5 varyant)</t>
   </si>
   <si>
@@ -393,7 +420,7 @@
     <t xml:space="preserve">Best-of-K, unit testlerle puanlanan</t>
   </si>
   <si>
-    <t xml:space="preserve">Yalnızca T0.3 Spearman ≥ 0.6 ise</t>
+    <t xml:space="preserve">Yalnızca T0.4 Spearman ≥ 0.6 ise</t>
   </si>
   <si>
     <t xml:space="preserve">Self-check'e göre gürültünün üstünde önde</t>
@@ -1081,7 +1108,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -1134,7 +1161,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -1159,24 +1186,24 @@
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>17</v>
@@ -1184,24 +1211,24 @@
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>17</v>
@@ -1211,22 +1238,22 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>17</v>
@@ -1234,24 +1261,24 @@
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>17</v>
@@ -1261,22 +1288,22 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>17</v>
@@ -1284,24 +1311,24 @@
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>33</v>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>17</v>
@@ -1311,22 +1338,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>17</v>
@@ -1336,22 +1363,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>17</v>
@@ -1359,24 +1386,24 @@
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>17</v>
@@ -1386,22 +1413,22 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>17</v>
@@ -1411,22 +1438,22 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>17</v>
@@ -1434,24 +1461,24 @@
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>17</v>
@@ -1459,24 +1486,24 @@
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>17</v>
@@ -1486,22 +1513,22 @@
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>17</v>
@@ -1511,22 +1538,22 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>17</v>
@@ -1536,22 +1563,22 @@
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>17</v>
@@ -1559,24 +1586,24 @@
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>17</v>
@@ -1584,24 +1611,24 @@
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>17</v>
@@ -1611,22 +1638,22 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>17</v>
@@ -1636,22 +1663,22 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>17</v>
@@ -1661,22 +1688,22 @@
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>17</v>
@@ -1686,22 +1713,22 @@
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>17</v>
@@ -1710,23 +1737,23 @@
       <c r="I27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>85</v>
+      <c r="A28" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>87</v>
+        <v>21</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>17</v>
@@ -1736,22 +1763,22 @@
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>71</v>
+        <v>97</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>17</v>
@@ -1761,22 +1788,22 @@
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="G30" s="6" t="s">
         <v>17</v>
@@ -1786,22 +1813,22 @@
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>17</v>
@@ -1809,24 +1836,24 @@
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>17</v>
@@ -1836,22 +1863,22 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>104</v>
+        <v>79</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>17</v>
@@ -1859,24 +1886,24 @@
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>17</v>
@@ -1886,22 +1913,22 @@
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>17</v>
@@ -1910,23 +1937,23 @@
       <c r="I35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>114</v>
+      <c r="A36" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>118</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>14</v>
+        <v>104</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>17</v>
@@ -1936,22 +1963,22 @@
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>17</v>
@@ -1959,24 +1986,24 @@
       <c r="H37" s="6"/>
       <c r="I37" s="6"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>122</v>
+        <v>21</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>17</v>
@@ -1986,22 +2013,22 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>71</v>
+        <v>132</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>17</v>
@@ -2009,24 +2036,24 @@
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
     </row>
-    <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>129</v>
+        <v>80</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="G40" s="6" t="s">
         <v>17</v>
@@ -2036,22 +2063,22 @@
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>71</v>
+        <v>138</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="G41" s="6" t="s">
         <v>17</v>
@@ -2059,24 +2086,24 @@
       <c r="H41" s="6"/>
       <c r="I41" s="6"/>
     </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>133</v>
+    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>135</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>17</v>
@@ -2086,22 +2113,22 @@
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>17</v>
@@ -2111,22 +2138,22 @@
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="G44" s="6" t="s">
         <v>17</v>
@@ -2136,22 +2163,22 @@
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>71</v>
+        <v>152</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>17</v>
@@ -2161,22 +2188,22 @@
     </row>
     <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>14</v>
+        <v>80</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="G46" s="6" t="s">
         <v>17</v>
@@ -2184,10 +2211,35 @@
       <c r="H46" s="6"/>
       <c r="I46" s="6"/>
     </row>
+    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H47" s="6"/>
+      <c r="I47" s="6"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I46"/>
+  <autoFilter ref="A4:I47"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G46" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G47" type="list">
       <formula1>"Bekliyor,Koşuyor,Bu sonuç çıktı,Bu sonuç çıkmadı,Atlandı"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2217,20 +2269,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2238,7 +2290,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2246,7 +2298,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2254,7 +2306,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -2282,12 +2334,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2295,7 +2347,7 @@
         <v>8</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2303,53 +2355,53 @@
         <v>17</v>
       </c>
       <c r="B5" s="12" t="n">
-        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$46,A5)</f>
-        <v>42</v>
+        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$47,A5)</f>
+        <v>43</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="B6" s="12" t="n">
-        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$46,A6)</f>
+        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$47,A6)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="B7" s="12" t="n">
-        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$46,A7)</f>
+        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$47,A7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="B8" s="12" t="n">
-        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$46,A8)</f>
+        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$47,A8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="B9" s="12" t="n">
-        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$46,A9)</f>
+        <f aca="false">COUNTIF('Test Planı'!$G$5:$G$47,A9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Test plan: gate vs current best, re-run wins, pairwise ranking, eval limits, time budget
</commit_message>
<xml_diff>
--- a/Test_Plani.xlsx
+++ b/Test_Plani.xlsx
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="174">
   <si>
     <t xml:space="preserve">Collections Builder — Test Planı ve Karar Kuralları</t>
   </si>
   <si>
-    <t xml:space="preserve">Kazanç = eşleştirilmiş case bazında testte p&lt;0.1 ve kritik case tiplerinde düşüş yok (aggregate 2×SD kullanılmaz). Sarı sütunlar ekip tarafından doldurulur (Durum açılır listeden).</t>
+    <t xml:space="preserve">Kazanç = MEVCUT EN İYİYE karşı eşleştirilmiş sign/Wilcoxon testte p&lt;0.1 + taze run tekrarında yön korunuyor + kritik case tiplerinde düşüş yok (düşüş de aynı testle). Sarı sütunlar ekip tarafından doldurulur (Durum açılır listeden).</t>
   </si>
   <si>
     <t xml:space="preserve">Bölüm</t>
@@ -72,7 +72,7 @@
     <t xml:space="preserve">Kickoff'tan önce</t>
   </si>
   <si>
-    <t xml:space="preserve">2–3 sahte brief, 7 tool + mock veri, 16 case tipi persona kütüphanesi, 4 kritik an unit testi hazır</t>
+    <t xml:space="preserve">5+ sahte brief (katı, Türkçe, plan yok dahil; farklı formatlar), 7 tool + mock veri, 16 case tipi persona kütüphanesi, 4 kritik an unit testi hazır</t>
   </si>
   <si>
     <t xml:space="preserve">Hazır değilse hiçbir test koşamaz; önce bu tamamlanır.</t>
@@ -102,19 +102,19 @@
     <t xml:space="preserve">T0.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Yargıç düzeltmesi (uyumdan önce)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool-call log verilir; eylemler sözlerden ayrı, evet/hayır sorular, sıcaklık 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uyum bu düzeltmeden sonra ölçülür.</t>
+    <t xml:space="preserve">Lokal yargıç = decision model (uyumdan önce kurulur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool-call log verilir; eylemler sözlerden ayrı; kontrol başına tek evet/hayır kararı; sıcaklık 0; sorular Policy'den üretilir; regex/phrase-match yok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uyum bu kurulumdan sonra ölçülür. Builder, kurallar izin vermedikçe değerlendirmede decision model'e bağımlı olmaz (sadece dev).</t>
   </si>
   <si>
     <t xml:space="preserve">T0.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Lokal yargıç ile Freya verdict uyumu (case tipi bazında)</t>
+    <t xml:space="preserve">Decision model yargıç ile Freya verdict uyumu (case tipi bazında)</t>
   </si>
   <si>
     <t xml:space="preserve">İlk practice verdict'leri dönünce</t>
@@ -135,18 +135,15 @@
     <t xml:space="preserve">T0.4</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit test skoru ile Freya skoru sıralaması (5 varyant)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spearman ≥ 0.6</t>
+    <t xml:space="preserve">Unit test skoru Freya ile aynı kazananı seçiyor mu? (≥8 A/B çifti, ikili sıralama uyumu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Çiftlerin ≥ %80'inde aynı kazanan</t>
   </si>
   <si>
     <t xml:space="preserve">Unit testler varyant eleme ve best-of-K puanlaması için kullanılır.</t>
   </si>
   <si>
-    <t xml:space="preserve">Spearman &lt; 0.6</t>
-  </si>
-  <si>
     <t xml:space="preserve">Unit testler yalnızca regresyon kontrolü olarak kalır.</t>
   </si>
   <si>
@@ -420,7 +417,7 @@
     <t xml:space="preserve">Best-of-K, unit testlerle puanlanan</t>
   </si>
   <si>
-    <t xml:space="preserve">Yalnızca T0.4 Spearman ≥ 0.6 ise</t>
+    <t xml:space="preserve">Yalnızca T0.4 ikili sıralama uyumu ≥ %80 ise ve değerlendirme süre sınırı izin veriyorsa</t>
   </si>
   <si>
     <t xml:space="preserve">Self-check'e göre gürültünün üstünde önde</t>
@@ -459,7 +456,7 @@
     <t xml:space="preserve">GEPA-lite, agent template'i üzerinde (Pareto: brief ve case tipi başına en iyi aday)</t>
   </si>
   <si>
-    <t xml:space="preserve">Yalnızca yargıç ≥ %85 ise</t>
+    <t xml:space="preserve">Yalnızca yargıç uyumu ≥ %90 ise (optimizer yargıcın kaçırdığını bulur)</t>
   </si>
   <si>
     <t xml:space="preserve">En iyi 3 aday Freya'da gürültünün üstünde önde, sahte brief'lerde düşüş yok</t>
@@ -507,7 +504,7 @@
     <t xml:space="preserve">Her değişiklik için kabul kapısı</t>
   </si>
   <si>
-    <t xml:space="preserve">Bir değişiklik ancak üç koşul birlikte sağlanırsa kalıcı olur. Yalnızca practice brief'te işe yarayan değişiklik reddedilir.</t>
+    <t xml:space="preserve">Bir değişiklik ancak dört koşul birlikte sağlanırsa kalıcı olur. Yalnızca practice brief'te işe yarayan değişiklik reddedilir.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -516,10 +513,13 @@
     <t xml:space="preserve">Koşul</t>
   </si>
   <si>
-    <t xml:space="preserve">Practice'te baseline'dan kötü değil.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En az 3 sahte brief'te düşüş yok.</t>
+    <t xml:space="preserve">Practice'te mevcut en iyiden kötü değil (eşleştirilmiş testle tanımlı düşüş yok) ve taze run tekrarında da öyle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5+ sahte brief'ten en az 3'ünde düşüş yok.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doymuş case'lerin kritik tiplerinde regresyon koşusu temiz.</t>
   </si>
   <si>
     <t xml:space="preserve">Builder tüm sahte brief'lerde hatasız agent üretiyor.</t>
@@ -1161,7 +1161,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -1211,7 +1211,7 @@
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
@@ -1325,10 +1325,10 @@
         <v>21</v>
       </c>
       <c r="E11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>17</v>
@@ -1338,22 +1338,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="C12" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>17</v>
@@ -1363,22 +1363,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="C13" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>44</v>
-      </c>
       <c r="E13" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>47</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>48</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>17</v>
@@ -1388,22 +1388,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>50</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>17</v>
@@ -1413,22 +1413,22 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>50</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>54</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>17</v>
@@ -1438,22 +1438,22 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>50</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E16" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>56</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>17</v>
@@ -1463,22 +1463,22 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E17" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>17</v>
@@ -1488,22 +1488,22 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>17</v>
@@ -1513,22 +1513,22 @@
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="F19" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>67</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>17</v>
@@ -1538,22 +1538,22 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="E20" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>17</v>
@@ -1563,22 +1563,22 @@
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>70</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>71</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E21" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>72</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>73</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>17</v>
@@ -1588,22 +1588,22 @@
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B22" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>70</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>71</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E22" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>75</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>17</v>
@@ -1613,22 +1613,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E23" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>79</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>17</v>
@@ -1638,22 +1638,22 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E24" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>81</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>17</v>
@@ -1663,22 +1663,22 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="F25" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>86</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>17</v>
@@ -1688,22 +1688,22 @@
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B26" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>84</v>
-      </c>
       <c r="E26" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G26" s="6" t="s">
         <v>17</v>
@@ -1713,22 +1713,22 @@
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B27" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>84</v>
-      </c>
       <c r="E27" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="F27" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>89</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>17</v>
@@ -1738,22 +1738,22 @@
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E28" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F28" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>92</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>17</v>
@@ -1763,22 +1763,22 @@
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B29" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="C29" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="E29" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="F29" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>17</v>
@@ -1788,22 +1788,22 @@
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="C30" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="D30" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>96</v>
-      </c>
       <c r="E30" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G30" s="6" t="s">
         <v>17</v>
@@ -1813,22 +1813,22 @@
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B31" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="C31" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="5" t="s">
-        <v>96</v>
-      </c>
       <c r="E31" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F31" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>17</v>
@@ -1838,22 +1838,22 @@
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B32" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="F32" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>106</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>17</v>
@@ -1863,22 +1863,22 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B33" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="D33" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E33" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>109</v>
-      </c>
       <c r="F33" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>17</v>
@@ -1888,22 +1888,22 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B34" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="D34" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E34" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="E34" s="5" t="s">
+      <c r="F34" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>17</v>
@@ -1913,22 +1913,22 @@
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B35" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E35" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="E35" s="5" t="s">
+      <c r="F35" s="5" t="s">
         <v>116</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>117</v>
       </c>
       <c r="G35" s="6" t="s">
         <v>17</v>
@@ -1938,22 +1938,22 @@
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B36" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="D36" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="E36" s="5" t="s">
+      <c r="F36" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>121</v>
       </c>
       <c r="G36" s="6" t="s">
         <v>17</v>
@@ -1963,22 +1963,22 @@
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B37" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="C37" s="5" t="s">
         <v>123</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E37" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="F37" s="5" t="s">
         <v>125</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>126</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>17</v>
@@ -1988,22 +1988,22 @@
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B38" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="C38" s="5" t="s">
         <v>123</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E38" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F38" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G38" s="6" t="s">
         <v>17</v>
@@ -2011,24 +2011,24 @@
       <c r="H38" s="6"/>
       <c r="I38" s="6"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B39" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="E39" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="F39" s="5" t="s">
         <v>132</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>133</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>17</v>
@@ -2036,24 +2036,24 @@
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B40" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="D40" s="5" t="s">
-        <v>131</v>
-      </c>
       <c r="E40" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G40" s="6" t="s">
         <v>17</v>
@@ -2063,22 +2063,22 @@
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B41" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="D41" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="E41" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="F41" s="5" t="s">
         <v>138</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>139</v>
       </c>
       <c r="G41" s="6" t="s">
         <v>17</v>
@@ -2088,22 +2088,22 @@
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B42" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D42" s="5" t="s">
-        <v>137</v>
-      </c>
       <c r="E42" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>17</v>
@@ -2113,22 +2113,22 @@
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B43" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B43" s="10" t="s">
+      <c r="C43" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="D43" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D43" s="5" t="s">
+      <c r="E43" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="E43" s="5" t="s">
+      <c r="F43" s="5" t="s">
         <v>145</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>146</v>
       </c>
       <c r="G43" s="6" t="s">
         <v>17</v>
@@ -2138,22 +2138,22 @@
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B44" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="C44" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="D44" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>144</v>
-      </c>
       <c r="E44" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="F44" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>148</v>
       </c>
       <c r="G44" s="6" t="s">
         <v>17</v>
@@ -2163,22 +2163,22 @@
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B45" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C45" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="D45" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="E45" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="F45" s="5" t="s">
         <v>152</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>153</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>17</v>
@@ -2188,22 +2188,22 @@
     </row>
     <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B46" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="D46" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D46" s="5" t="s">
-        <v>151</v>
-      </c>
       <c r="E46" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G46" s="6" t="s">
         <v>17</v>
@@ -2213,22 +2213,22 @@
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B47" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C47" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="D47" s="5" t="s">
         <v>156</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>157</v>
       </c>
       <c r="E47" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>17</v>
@@ -2260,7 +2260,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2269,20 +2269,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>161</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2290,7 +2290,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2298,7 +2298,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2306,6 +2306,14 @@
         <v>3</v>
       </c>
       <c r="B7" s="12" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>165</v>
       </c>
     </row>

</xml_diff>